<commit_message>
Modificacion grande de eis_pip, ahora exporta metadatos, datos con suss respectivas unidades
</commit_message>
<xml_diff>
--- a/outputs/EISPOT_0V_2_#1.xlsx
+++ b/outputs/EISPOT_0V_2_#1.xlsx
@@ -423,29 +423,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Field</t>
+          <t>Campo</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Técnica</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -453,11 +459,12 @@
           <t>Potentiostatic EIS</t>
         </is>
       </c>
+      <c r="C2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -465,11 +472,12 @@
           <t>24/2/2026</t>
         </is>
       </c>
+      <c r="C3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Hora</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -477,6 +485,7 @@
           <t>0:22:55</t>
         </is>
       </c>
+      <c r="C4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -487,55 +496,85 @@
       <c r="B5" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>freqinit</t>
+          <t>Frecuencia inicial</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>100000</v>
       </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Hz</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>freqfinal</t>
+          <t>Frecuencia final</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
         <v>1000</v>
       </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Hz</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ptsperdec</t>
+          <t>Puntos por década</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>points/decade</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>vac</t>
+          <t>Amplitud</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>mV rms</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>Área</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
         <v>25</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>cm^2</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -549,11 +588,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -572,7 +611,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Frequency</t>
+          <t>Frecuencia</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -612,679 +651,727 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Temperature</t>
+          <t>Temperatura</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>100078.1</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>0.0140985</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>0.0059622</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>0.0153074</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>22.9232</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>-0.0025679</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0.3414271</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>62.38431</v>
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Hz</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ohm</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ohm</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ohm</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>79453.13</v>
+        <v>100078.1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.0139613</v>
+        <v>0.0140985</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.0048196</v>
+        <v>0.0059622</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.0147698</v>
+        <v>0.0153074</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>19.04506</v>
+        <v>22.9232</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>-0.0014785</v>
+        <v>-0.0025679</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>0.3414339</v>
+        <v>0.3414271</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>62.37391</v>
+        <v>62.38431</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>63140.62</v>
+        <v>79453.13</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.0138486</v>
+        <v>0.0139613</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.0038948</v>
+        <v>0.0048196</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.0143859</v>
+        <v>0.0147698</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>15.70819</v>
+        <v>19.04506</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>-0.00263</v>
+        <v>-0.0014785</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>0.3414341</v>
+        <v>0.3414339</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>62.40363</v>
+        <v>62.37391</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>50203.12</v>
+        <v>63140.62</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.0137487</v>
+        <v>0.0138486</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.0031424</v>
+        <v>0.0038948</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.0141033</v>
+        <v>0.0143859</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12.87432</v>
+        <v>15.70819</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>-0.0016665</v>
+        <v>-0.00263</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0.3414395</v>
+        <v>0.3414341</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>62.38742</v>
+        <v>62.40363</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>39890.62</v>
+        <v>50203.12</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.0136741</v>
+        <v>0.0137487</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.0025183</v>
+        <v>0.0031424</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.013904</v>
+        <v>0.0141033</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>10.43503</v>
+        <v>12.87432</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>-0.0020762</v>
+        <v>-0.0016665</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0.3414391</v>
+        <v>0.3414395</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>62.38379</v>
+        <v>62.38742</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>31640.63</v>
+        <v>39890.62</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.0136097</v>
+        <v>0.0136741</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.0020042</v>
+        <v>0.0025183</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.0137564</v>
+        <v>0.013904</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>8.377141999999999</v>
+        <v>10.43503</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>-0.0022292</v>
+        <v>-0.0020762</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.341434</v>
+        <v>0.3414391</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>62.38073</v>
+        <v>62.38379</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>25171.88</v>
+        <v>31640.63</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.0135675</v>
+        <v>0.0136097</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.0015861</v>
+        <v>0.0020042</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.0136599</v>
+        <v>0.0137564</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>6.667912</v>
+        <v>8.377141999999999</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>-0.0024219</v>
+        <v>-0.0022292</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>0.3414329</v>
+        <v>0.341434</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>62.38298</v>
+        <v>62.38073</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>20015.62</v>
+        <v>25171.88</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.0135387</v>
+        <v>0.0135675</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.0012453</v>
+        <v>0.0015861</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.0135959</v>
+        <v>0.0136599</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>5.255154</v>
+        <v>6.667912</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>-0.0029743</v>
+        <v>-0.0024219</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0.3414359</v>
+        <v>0.3414329</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>62.39997</v>
+        <v>62.38298</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>15890.62</v>
+        <v>20015.62</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.013524</v>
+        <v>0.0135387</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.0009592</v>
+        <v>0.0012453</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.013558</v>
+        <v>0.0135959</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>4.057134</v>
+        <v>5.255154</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>-0.0026796</v>
+        <v>-0.0029743</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>0.3414345</v>
+        <v>0.3414359</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>62.38594</v>
+        <v>62.39997</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>12609.38</v>
+        <v>15890.62</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.0135104</v>
+        <v>0.013524</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.0007219</v>
+        <v>0.0009592</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.0135297</v>
+        <v>0.013558</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>3.058671</v>
+        <v>4.057134</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>-0.0024853</v>
+        <v>-0.0026796</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>0.3414396</v>
+        <v>0.3414345</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>62.40276</v>
+        <v>62.38594</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>10078.13</v>
+        <v>12609.38</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.0135049</v>
+        <v>0.0135104</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.0005241</v>
+        <v>0.0007219</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.013515</v>
+        <v>0.0135297</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>2.222245</v>
+        <v>3.058671</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>-0.0033788</v>
+        <v>-0.0024853</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0.3414367</v>
+        <v>0.3414396</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>62.37671</v>
+        <v>62.40276</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>8015.625</v>
+        <v>10078.13</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.0135067</v>
+        <v>0.0135049</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.0003518</v>
+        <v>0.0005241</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.0135113</v>
+        <v>0.013515</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>1.491875</v>
+        <v>2.222245</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>-0.0032693</v>
+        <v>-0.0033788</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0.3414341</v>
+        <v>0.3414367</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>62.3937</v>
+        <v>62.37671</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>6328.125</v>
+        <v>8015.625</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.0135174</v>
+        <v>0.0135067</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.0001936</v>
+        <v>0.0003518</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.0135188</v>
+        <v>0.0135113</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.8206955</v>
+        <v>1.491875</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>-0.0031275</v>
+        <v>-0.0032693</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>0.3414359</v>
+        <v>0.3414341</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>62.40042</v>
+        <v>62.3937</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>5015.625</v>
+        <v>6328.125</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.0135316</v>
+        <v>0.0135174</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>6.007775e-05</v>
+        <v>0.0001936</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.0135317</v>
+        <v>0.0135188</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.2543816</v>
+        <v>0.8206955</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>-0.0032598</v>
+        <v>-0.0031275</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0.3414348</v>
+        <v>0.3414359</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>62.39809</v>
+        <v>62.40042</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>3984.375</v>
+        <v>5015.625</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.0135465</v>
+        <v>0.0135316</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-6.481124e-05</v>
+        <v>6.007775e-05</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.0135466</v>
+        <v>0.0135317</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>-0.2741214</v>
+        <v>0.2543816</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>-0.0033302</v>
+        <v>-0.0032598</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0.3414368</v>
+        <v>0.3414348</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>62.39874</v>
+        <v>62.39809</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>3170.956</v>
+        <v>3984.375</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.0135702</v>
+        <v>0.0135465</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-0.0001868</v>
+        <v>-6.481124e-05</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.0135715</v>
+        <v>0.0135466</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>-0.7885715</v>
+        <v>-0.2741214</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>-0.0033298</v>
+        <v>-0.0033302</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0.3414379</v>
+        <v>0.3414368</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>62.39771</v>
+        <v>62.39874</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>2527.573</v>
+        <v>3170.956</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.0136007</v>
+        <v>0.0135702</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-0.0003081</v>
+        <v>-0.0001868</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0.0136042</v>
+        <v>0.0135715</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>-1.2979</v>
+        <v>-0.7885715</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>-0.0038077</v>
+        <v>-0.0033298</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0.3414333</v>
+        <v>0.3414379</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>62.39754</v>
+        <v>62.39771</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1976.103</v>
+        <v>2527.573</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.0136385</v>
+        <v>0.0136007</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>-0.0004451</v>
+        <v>-0.0003081</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0.0136458</v>
+        <v>0.0136042</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>-1.869123</v>
+        <v>-1.2979</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>-0.0029144</v>
+        <v>-0.0038077</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0.3414378</v>
+        <v>0.3414333</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>62.39402</v>
+        <v>62.39754</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1577.524</v>
+        <v>1976.103</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.0136853</v>
+        <v>0.0136385</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-0.0005798</v>
+        <v>-0.0004451</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0.0136976</v>
+        <v>0.0136458</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>-2.426179</v>
+        <v>-1.869123</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>-0.0031066</v>
+        <v>-0.0029144</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0.3414384</v>
+        <v>0.3414378</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>62.40379</v>
+        <v>62.39402</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>1265.625</v>
+        <v>1577.524</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.0137362</v>
+        <v>0.0136853</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-0.0007243</v>
+        <v>-0.0005798</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.0137553</v>
+        <v>0.0136976</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>-3.018498</v>
+        <v>-2.426179</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>-0.0034504</v>
+        <v>-0.0031066</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>0.3414393</v>
+        <v>0.3414384</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>62.41189</v>
+        <v>62.40379</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>1265.625</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>0.0137362</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>-0.0007243</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0.0137553</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>-3.018498</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>-0.0034504</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0.3414393</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>62.41189</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>998.264</v>
       </c>
-      <c r="C22" s="2" t="n">
+      <c r="C23" s="2" t="n">
         <v>0.0137987</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D23" s="2" t="n">
         <v>-0.0009033999999999999</v>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="2" t="n">
+      <c r="E23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="n">
         <v>0.0138283</v>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>-3.745814</v>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>-0.003608</v>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I23" s="2" t="n">
         <v>0.3414375</v>
       </c>
-      <c r="J22" s="2" t="n">
+      <c r="J23" s="2" t="n">
         <v>62.42235</v>
       </c>
     </row>

</xml_diff>